<commit_message>
Rename rtf_plan() / class rtf_plan to table_plan (0.0.7)
The plan lives in tflspec, not rtfreporter, and is the table-building
plan paired with table_spec, so it drops rtfreporter's rtf_ prefix:
table_plan() returns an object of class table_plan (print and
as_rtftables methods follow).  rtf_plan() is kept as the same function
under its former name (superseded, no warning), so existing programs
run unchanged.  plan_template() writes table_plan(); the bundled
example workbooks' _README sheets are regenerated (only that text
changed; the five reports' RTF are byte-identical).

Closes #7

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -399,7 +399,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
+          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。table_plan(data; spec = read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。table_plan(data; spec = read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Give every export the tfl_ prefix (0.0.9)
tflspec is attached with cards/cardx (ard_*) and rtfreporter (rtf_*);
a package-wide prefix keeps its names from colliding on library() and
says whose function it is, mirroring rtfreporter's rtf_.  Scheme:
tfl_ + area (ard, table, plan, report, listing, fig, plot) + action.
The pp_ (plotplanner) names and the plot/fig mix go away; S3 classes
follow (tfl_plan, tfl_table_spec, tfl_fig_spec, tfl_code, ...).

Every former name is kept in R/superseded.R as the same function
(superseded, no warning, one internal help page with the old -> new
table), so existing programs and tflplanner run unchanged; a test
checks each alias is identical to exactly one tfl_ function.

Generated code writes the new names; the bundled example workbooks'
_README sheets are regenerated (names only); the five example reports'
RTF (from code and from spec) are byte-identical to before the rename.

Closes #9

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -399,7 +399,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。table_plan(data; spec = read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
+          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。tfl_plan(data; spec = tfl_read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。table_plan(data; spec = read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。tfl_plan(data; spec = tfl_read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
+          <t>tfl_plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
+          <t>tfl_plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>group_page = TRUE で group_col の値ごとに改ページ（plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
+          <t>group_page = TRUE で group_col の値ごとに改ページ（tfl_plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>plan_blanks() の where / first / last / counted。</t>
+          <t>tfl_plan_blanks() の where / first / last / counted。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>plan_stub() の vars / into / indent / group_summary / before。</t>
+          <t>tfl_plan_stub() の vars / into / indent / group_summary / before。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
+          <t>tfl_plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>以下は表の周りの定義。read_report_spec(c(report.xlsx; tables.xlsx); output_id = ) で 1 冊でも分冊でも読める。同じシートに行があるのは 1 冊だけにする（空のシートと study は重なってよい）。rtf_report(spec; plan) で rtf_document、report_path(spec) で出力先。</t>
+          <t>以下は表の周りの定義。tfl_read_report_spec(c(report.xlsx; tables.xlsx); output_id = ) で 1 冊でも分冊でも読める。同じシートに行があるのは 1 冊だけにする（空のシートと study は重なってよい）。tfl_report(spec; plan) で rtf_document、tfl_report_path(spec) で出力先。</t>
         </is>
       </c>
     </row>

</xml_diff>